<commit_message>
In case of data not available for AP Voucher data will be created using api calls (AR Voucher for non supplier type and Service Invoice Adhoc for supplier type).After that test will be continued.Report for PreRequisite data creation needs to be improved.
</commit_message>
<xml_diff>
--- a/src/test/resources/UsersList.xlsx
+++ b/src/test/resources/UsersList.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="20490" windowHeight="7620"/>
+    <workbookView windowWidth="19890" windowHeight="7500"/>
   </bookViews>
   <sheets>
     <sheet name="UIUsers" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="20">
   <si>
     <t>username</t>
   </si>
@@ -55,6 +55,15 @@
   </si>
   <si>
     <t>mk</t>
+  </si>
+  <si>
+    <t>webapi1</t>
+  </si>
+  <si>
+    <t>webapi2</t>
+  </si>
+  <si>
+    <t>webapi3</t>
   </si>
   <si>
     <t>APIKey</t>
@@ -1224,8 +1233,8 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:B5"/>
-  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelRow="4" outlineLevelCol="1"/>
+  <dimension ref="A1:B8"/>
+  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelRow="7" outlineLevelCol="1"/>
   <cols>
     <col min="1" max="1" width="13" style="1" customWidth="1"/>
     <col min="2" max="2" width="11.2190476190476" style="1" customWidth="1"/>
@@ -1269,6 +1278,30 @@
       </c>
       <c r="B5" s="1" t="s">
         <v>8</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2">
+      <c r="A6" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2">
+      <c r="A7" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2">
+      <c r="A8" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>11</v>
       </c>
     </row>
   </sheetData>
@@ -1288,34 +1321,34 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="B1" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
     </row>
     <row r="2" spans="1:2">
       <c r="A2" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="B2" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
     </row>
     <row r="3" spans="1:2">
       <c r="A3" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="B3" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="B4" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
General Voucher Bug Fixes 11. COMBO-09 — picker opens, option click doesn't commit. 12. HEADER-03/DELETE-01 — Actions→Edit/Delete still disabled. 13. EDIT-DETAIL — logging invisible in the HTML report.
</commit_message>
<xml_diff>
--- a/src/test/resources/UsersList.xlsx
+++ b/src/test/resources/UsersList.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="18">
   <si>
     <t>username</t>
   </si>
@@ -58,12 +58,6 @@
   </si>
   <si>
     <t>webapi3</t>
-  </si>
-  <si>
-    <t>barbara</t>
-  </si>
-  <si>
-    <t>bt</t>
   </si>
   <si>
     <t>APIKey</t>
@@ -1233,8 +1227,8 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:B8"/>
-  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelRow="7" outlineLevelCol="1"/>
+  <dimension ref="A1:B7"/>
+  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelRow="6" outlineLevelCol="1"/>
   <cols>
     <col min="1" max="1" width="13" style="1" customWidth="1"/>
     <col min="2" max="2" width="11.2190476190476" style="1" customWidth="1"/>
@@ -1294,14 +1288,6 @@
       </c>
       <c r="B7" s="1" t="s">
         <v>9</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2">
-      <c r="A8" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B8" s="1" t="s">
-        <v>11</v>
       </c>
     </row>
   </sheetData>
@@ -1321,34 +1307,34 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B1" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="2" spans="1:2">
       <c r="A2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B2" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="3" spans="1:2">
       <c r="A3" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B3" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B4" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
     </row>
   </sheetData>

</xml_diff>